<commit_message>
Agregar 6 productos nuevos: papel higienico convencional y rollos multiuso
C.6602 C.6607 C.6122 C.6616 (papel higienico) y C.6648 C.6639 (bobinas multiuso)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/precios.xlsx
+++ b/precios.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -587,10 +587,6 @@
           <t xml:space="preserve">  Toallas en Rollo</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n"/>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="10" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -723,10 +719,6 @@
           <t xml:space="preserve">  Toallas Intercaladas</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="10" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -845,22 +837,22 @@
           <t>201010103</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>C.6112</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Elite Plus Higienico Jumbo SH 300M x4</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>pack (4 rollos)</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" t="n">
         <v>14950</v>
       </c>
     </row>
@@ -915,95 +907,109 @@
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Bobinas</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="10" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>6602</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C.6602</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Elite Plus Higienico SH 30M x48</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>bolson (48 rollos)</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>18530</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>204010108</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>C.6264</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Elite Plus Bobina DH Industrial 400M x2</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>par (2 bobinas)</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>31730</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>6607</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>C.6607</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Elite Plus Higienico SH 50M x48</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>bolson (48 rollos)</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>26330</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>608010547</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>C.6213</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Elite Excellence Bobina DH 200M x2 (1000 usos)</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>par (2 bobinas)</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>15280</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>6122</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>C.6122</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Elite Plus Higienico SH 100M x40</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>bolson (40 rollos)</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>44660</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>608020000</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>C.6214</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Elite Classic Bobina SH Industrial 400M x2</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>par (2 bobinas)</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n">
-        <v>36210</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>6616</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>C.6616</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Elite Excellence Higienico DH 30M x40</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>bolson (40 rollos)</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>24320</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Servilletas</t>
+          <t xml:space="preserve">  Bobinas</t>
         </is>
       </c>
       <c r="B23" s="9" t="n"/>
@@ -1014,276 +1020,401 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>203010104</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>C.6567</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Elite Plus Servilleta SH Blanca 1000u 30x30</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>caja (1.000 unidades)</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>12550</v>
+          <t>204010108</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>C.6264</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Elite Plus Bobina DH Industrial 400M x2</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>par (2 bobinas)</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>31730</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>608020016</t>
+          <t>608010547</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>C.6523</t>
+          <t>C.6213</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Elite Classic Servilleta Intercalada 10x21 250x72</t>
+          <t>Elite Excellence Bobina DH 200M x2 (1000 usos)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>caja (72 paquetes x 250u)</t>
+          <t>par (2 bobinas)</t>
         </is>
       </c>
       <c r="E25" s="8" t="n">
-        <v>75820</v>
+        <v>15280</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>608020017</t>
+          <t>608020000</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>C.6540</t>
+          <t>C.6214</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Elite Classic Servilleta Fast Food 16.5x20 350x24</t>
+          <t>Elite Classic Bobina SH Industrial 400M x2</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>caja (24 paquetes x 350u)</t>
+          <t>par (2 bobinas)</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>48570</v>
+        <v>36210</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Paños</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="10" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>6648</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C.6648</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Elite Plus Rollo Multiuso DH 50 Panos x30</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>caja (30 rollos)</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>17090</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>608020066</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>C.6389</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Maxwipe Max 50 - 690 panos</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>unidad (690 panos)</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="n">
-        <v>51780</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>6639</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>C.6639</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Elite Excellence Rollo Multiuso DH 200 Panos x12</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>bolson (12 rollos)</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>23430</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>608020085</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>C.6384</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Maxwipe Max 60 - 890 panos</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>unidad (890 panos)</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="n">
-        <v>92240</v>
-      </c>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Servilletas</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="n"/>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="10" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>608020086</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>C.6385</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Maxwipe Max 60 Estuche 50u x12</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>caja (12 estuches x 50u)</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n">
-        <v>83880</v>
+          <t>203010104</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>C.6567</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Elite Plus Servilleta SH Blanca 1000u 30x30</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>caja (1.000 unidades)</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="n">
+        <v>12550</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>608020087</t>
+          <t>608020016</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>C.6386</t>
+          <t>C.6523</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Maxwipe Max 70 - 750 panos</t>
+          <t>Elite Classic Servilleta Intercalada 10x21 250x72</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>unidad (750 panos)</t>
+          <t>caja (72 paquetes x 250u)</t>
         </is>
       </c>
       <c r="E31" s="8" t="n">
-        <v>104730</v>
+        <v>75820</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>608020088</t>
+          <t>608020017</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>C.6388</t>
+          <t>C.6540</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Maxwipe Max 80 Blanco 80u x6</t>
+          <t>Elite Classic Servilleta Fast Food 16.5x20 350x24</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>caja (6 packs x 80u) - Blanco</t>
+          <t>caja (24 paquetes x 350u)</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>127350</v>
+        <v>48570</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>608020089</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>C.6387</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Maxwipe Max 80 Azul 80u x6</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>caja (6 packs x 80u) - Azul</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="n">
-        <v>144020</v>
-      </c>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Paños</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="9" t="n"/>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
+          <t>608020066</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>C.6389</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Maxwipe Max 50 - 690 panos</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>unidad (690 panos)</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="n">
+        <v>51780</v>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>608020085</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>C.6384</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Maxwipe Max 60 - 890 panos</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>unidad (890 panos)</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="n">
+        <v>92240</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>608020086</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>C.6385</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Maxwipe Max 60 Estuche 50u x12</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>caja (12 estuches x 50u)</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>83880</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>608020087</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>C.6386</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Maxwipe Max 70 - 750 panos</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>unidad (750 panos)</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>104730</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>608020088</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>C.6388</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Maxwipe Max 80 Blanco 80u x6</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>caja (6 packs x 80u) - Blanco</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>127350</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>608020089</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>C.6387</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Maxwipe Max 80 Azul 80u x6</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>caja (6 packs x 80u) - Azul</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>144020</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
           <t>608020090</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>C.6286</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>Maxwipe Max 70 88u x6</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>caja (6 packs x 88u)</t>
         </is>
       </c>
-      <c r="E34" s="6" t="n">
+      <c r="E40" s="6" t="n">
         <v>118980</v>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar precios Elite 08/06/2026 (18 productos)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/precios.xlsx
+++ b/precios.xlsx
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>23580</v>
+        <v>25070</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>20290</v>
+        <v>21570</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>24980</v>
+        <v>26550</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>19510</v>
+        <v>20740</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>24760</v>
+        <v>26320</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>26820</v>
+        <v>28510</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>87170</v>
+        <v>92670</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="E17" s="8" t="n">
-        <v>24400</v>
+        <v>25940</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>18530</v>
+        <v>19700</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>26330</v>
+        <v>27990</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>44660</v>
+        <v>47470</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>24320</v>
+        <v>25850</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="E25" s="8" t="n">
-        <v>15280</v>
+        <v>26320</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>36210</v>
+        <v>38500</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>17090</v>
+        <v>18170</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>23430</v>
+        <v>24900</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="E31" s="8" t="n">
-        <v>75820</v>
+        <v>80600</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>48570</v>
+        <v>51640</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">

</xml_diff>